<commit_message>
Add linked mini income statement & balance sheet (auto-fed from project simulator)
</commit_message>
<xml_diff>
--- a/Hennecke/candidacy/Simulatore_Margine_Commessa.xlsx
+++ b/Hennecke/candidacy/Simulatore_Margine_Commessa.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Margine Commessa" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CE &amp; SP" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -100,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -150,6 +151,30 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1194,4 +1219,358 @@
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:F25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="3" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="17" t="inlineStr">
+        <is>
+          <t>Mini Conto Economico &amp; Stato Patrimoniale — collegati alla commessa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="18" t="inlineStr">
+        <is>
+          <t>Si aggiornano in automatico al variare degli input del foglio 'Margine Commessa'. Importi in € migliaia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>CONTO ECONOMICO — a commessa, cumulato a oggi</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>STATO PATRIMONIALE — a oggi</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>A) Valore della produzione</t>
+        </is>
+      </c>
+      <c r="E5" s="20" t="inlineStr">
+        <is>
+          <t>INPUT: Capitale iniziale / PN (cassa apportata)</t>
+        </is>
+      </c>
+      <c r="F5" s="21" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Ricavi (SAL fatturati)</t>
+        </is>
+      </c>
+      <c r="C6" s="22">
+        <f>'Margine Commessa'!C9</f>
+        <v/>
+      </c>
+      <c r="E6" s="19" t="inlineStr">
+        <is>
+          <t>ATTIVO</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Variazione lavori in corso su ordinazione</t>
+        </is>
+      </c>
+      <c r="C7" s="22">
+        <f>'Margine Commessa'!C22-'Margine Commessa'!C9</f>
+        <v/>
+      </c>
+      <c r="E7" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Cassa</t>
+        </is>
+      </c>
+      <c r="F7" s="22">
+        <f>F5+'Margine Commessa'!C10-'Margine Commessa'!C7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Totale valore della produzione</t>
+        </is>
+      </c>
+      <c r="C8" s="23">
+        <f>C6+C7</f>
+        <v/>
+      </c>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Lavori in corso su ordinazione (WIP / contract asset)</t>
+        </is>
+      </c>
+      <c r="F8" s="22">
+        <f>MAX('Margine Commessa'!C22-'Margine Commessa'!C9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>B) Costi della produzione</t>
+        </is>
+      </c>
+      <c r="E9" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Crediti v/clienti</t>
+        </is>
+      </c>
+      <c r="F9" s="22">
+        <f>MAX('Margine Commessa'!C9-'Margine Commessa'!C10,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Costi di commessa (materie/servizi/personale)</t>
+        </is>
+      </c>
+      <c r="C10" s="22">
+        <f>'Margine Commessa'!C7</f>
+        <v/>
+      </c>
+      <c r="E10" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   TOTALE ATTIVO</t>
+        </is>
+      </c>
+      <c r="F10" s="23">
+        <f>F7+F8+F9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Accantonamento perdita attesa su commessa</t>
+        </is>
+      </c>
+      <c r="C11" s="22">
+        <f>IF('Margine Commessa'!C19&lt;0,'Margine Commessa'!C24-'Margine Commessa'!C19,0)</f>
+        <v/>
+      </c>
+      <c r="E11" s="19" t="inlineStr">
+        <is>
+          <t>PASSIVO E PATRIMONIO NETTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Totale costi della produzione</t>
+        </is>
+      </c>
+      <c r="C12" s="23">
+        <f>C10+C11</f>
+        <v/>
+      </c>
+      <c r="E12" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Capitale iniziale</t>
+        </is>
+      </c>
+      <c r="F12" s="22">
+        <f>F5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>RISULTATO OPERATIVO (EBIT)</t>
+        </is>
+      </c>
+      <c r="C13" s="23">
+        <f>C8-C12</f>
+        <v/>
+      </c>
+      <c r="E13" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Risultato d'esercizio</t>
+        </is>
+      </c>
+      <c r="F13" s="22">
+        <f>C15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   EBIT margin %</t>
+        </is>
+      </c>
+      <c r="C14" s="24">
+        <f>IF(C8=0,0,C13/C8)</f>
+        <v/>
+      </c>
+      <c r="E14" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Patrimonio netto</t>
+        </is>
+      </c>
+      <c r="F14" s="25">
+        <f>F12+F13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>RISULTATO D'ESERCIZIO (ante imposte)</t>
+        </is>
+      </c>
+      <c r="C15" s="23">
+        <f>C13</f>
+        <v/>
+      </c>
+      <c r="E15" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Fondo rischi e oneri (perdita su commessa)</t>
+        </is>
+      </c>
+      <c r="F15" s="22">
+        <f>C11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="E16" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Anticipi da clienti (contract liability)</t>
+        </is>
+      </c>
+      <c r="F16" s="22">
+        <f>MAX('Margine Commessa'!C9-'Margine Commessa'!C22,0)+MAX('Margine Commessa'!C10-'Margine Commessa'!C9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="E17" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   TOTALE PASSIVO E PN</t>
+        </is>
+      </c>
+      <c r="F17" s="23">
+        <f>F14+F15+F16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="E18" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Quadratura (Attivo − Passivo)</t>
+        </is>
+      </c>
+      <c r="F18" s="25">
+        <f>F10-F17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="26" t="inlineStr">
+        <is>
+          <t>Logica e ipotesi (didattiche):</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>• Ricavi a CE = prezzo × % completamento (POC). La differenza tra ricavi maturati e fatturato alimenta i Lavori in corso (attivo) o gli Anticipi (passivo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>• Se la commessa è in perdita (EAC &gt; prezzo), l'intera perdita attesa è accantonata subito (Fondo rischi) → vedi voce CE 'Accantonamento'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>• Lo Stato Patrimoniale QUADRA sempre (cella F18 = 0): è costruito in doppia partita a partire dalla commessa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t>• Ipotesi semplificatrici: costi tutti pagati per cassa, nessun debito v/fornitori, nessuna imposta/onere finanziario. Scopo solo didattico.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>• Prova: nel foglio 'Margine Commessa' porta i Costi a finire (C8) a 6.300 → la commessa va in perdita → EBIT negativo e nasce il Fondo rischi.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="B21:F21"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="B24:F24"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="B25:F25"/>
+    <mergeCell ref="B23:F23"/>
+    <mergeCell ref="B1:F1"/>
+    <mergeCell ref="B22:F22"/>
+    <mergeCell ref="B4:C4"/>
+  </mergeCells>
+  <conditionalFormatting sqref="F18">
+    <cfRule type="expression" priority="1" dxfId="4">
+      <formula>ABS(F18)&lt;0.01</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="2">
+      <formula>ABS(F18)&gt;=0.01</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C13">
+    <cfRule type="expression" priority="3" dxfId="1">
+      <formula>C13&lt;0</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="0">
+      <formula>C13&gt;=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>